<commit_message>
label Table S4 as the primary top-500 analysis
</commit_message>
<xml_diff>
--- a/reference_results/supplementary_tables/Supplementary_Table_S4_statistical_tests_top500_markers.xlsx
+++ b/reference_results/supplementary_tables/Supplementary_Table_S4_statistical_tests_top500_markers.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="59">
   <si>
-    <t>Top-500 marker-set sensitivity analysis</t>
+    <t>Supplementary Table S4. Statistical comparisons of predictive ability among models and between marker panels (primary top-500 analysis)</t>
   </si>
   <si>
-    <t>Top-500 sensitivity analysis: statistical comparison of predictive ability among M1, M2, M3 and M4-500 and between marker panels, by trait and cross-validation scheme.</t>
+    <t>Primary top-500 analysis: statistical comparison of predictive ability among M1, M2, M3 and M4-500 and between marker panels, by trait and cross-validation scheme.</t>
   </si>
   <si>
     <t>Sheet</t>

</xml_diff>